<commit_message>
KPI_Historico actualizado — Abr-2026
</commit_message>
<xml_diff>
--- a/Tablas/KPI_Historico.xlsx
+++ b/Tablas/KPI_Historico.xlsx
@@ -1,34 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CLAUDE_CODE\MONITOR_DE_GESTION\outputs\2026_03\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7718CB6-CBE3-4AD6-B4C3-D925C228F3F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="3240" yWindow="3420" windowWidth="21660" windowHeight="13157" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -65,14 +46,14 @@
     <t>Mar-2026</t>
   </si>
   <si>
-    <t>|</t>
+    <t>Abr-2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -109,14 +90,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -404,11 +377,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -425,12 +398,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2">
-        <v>0.57999999999999996</v>
+        <v>0.58</v>
       </c>
       <c r="C2">
         <v>0.76</v>
@@ -439,10 +412,10 @@
         <v>0.49</v>
       </c>
       <c r="E2">
-        <v>0.69499999999999995</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+        <v>0.695</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -456,10 +429,10 @@
         <v>0.36</v>
       </c>
       <c r="E3">
-        <v>0.65449999999999997</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+        <v>0.6545</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -473,10 +446,10 @@
         <v>0.44</v>
       </c>
       <c r="E4">
-        <v>0.70199999999999996</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+        <v>0.702</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -490,32 +463,44 @@
         <v>0.59</v>
       </c>
       <c r="E5">
-        <v>0.63550000000000006</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+        <v>0.6355000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>9</v>
       </c>
       <c r="B6">
-        <v>0.61399999999999999</v>
+        <v>0.614</v>
       </c>
       <c r="C6">
-        <v>0.67500000000000004</v>
+        <v>0.675</v>
       </c>
       <c r="D6">
-        <v>0.50600000000000001</v>
+        <v>0.506</v>
       </c>
       <c r="E6">
-        <v>0.61375000000000002</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="D10" t="s">
+        <v>0.61375</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
         <v>10</v>
       </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0.7354000000000001</v>
+      </c>
+      <c r="D7">
+        <v>0.31</v>
+      </c>
+      <c r="E7">
+        <v>0.3194</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: KPI_Historico actualizado abril 2026
</commit_message>
<xml_diff>
--- a/Tablas/KPI_Historico.xlsx
+++ b/Tablas/KPI_Historico.xlsx
@@ -1,70 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>Mes</t>
-  </si>
-  <si>
-    <t>Satisfacción</t>
-  </si>
-  <si>
-    <t>Cierre</t>
-  </si>
-  <si>
-    <t>SLA</t>
-  </si>
-  <si>
-    <t>Score KPI</t>
-  </si>
-  <si>
-    <t>Nov-2025</t>
-  </si>
-  <si>
-    <t>Dic-2025</t>
-  </si>
-  <si>
-    <t>Ene-2026</t>
-  </si>
-  <si>
-    <t>Feb-2026</t>
-  </si>
-  <si>
-    <t>Mar-2026</t>
-  </si>
-  <si>
-    <t>Abr-2026</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -83,13 +46,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -377,127 +407,153 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Satisfacción</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Cierre</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>SLA</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Score KPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Nov-2025</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>0.58</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>0.76</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>0.49</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>0.695</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Dic-2025</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>0.54</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>0.75</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>0.36</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>0.6545</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ene-2026</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>0.61</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>0.88</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>0.44</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>0.702</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Feb-2026</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>0.59</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>0.72</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>0.59</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>0.6355000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Mar-2026</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>0.614</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>0.675</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>0.506</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>0.61375</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>0.6318</v>
-      </c>
-      <c r="C7">
-        <v>0.7354000000000001</v>
-      </c>
-      <c r="D7">
-        <v>0.31</v>
-      </c>
-      <c r="E7">
-        <v>0.6036899999999999</v>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Abr-2026</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.6294999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KPI_Historico actualizado v2 - Abr-2026
</commit_message>
<xml_diff>
--- a/Tablas/KPI_Historico.xlsx
+++ b/Tablas/KPI_Historico.xlsx
@@ -1,33 +1,70 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+  <si>
+    <t>Mes</t>
+  </si>
+  <si>
+    <t>Satisfacción</t>
+  </si>
+  <si>
+    <t>Cierre</t>
+  </si>
+  <si>
+    <t>SLA</t>
+  </si>
+  <si>
+    <t>Score KPI</t>
+  </si>
+  <si>
+    <t>Nov-2025</t>
+  </si>
+  <si>
+    <t>Dic-2025</t>
+  </si>
+  <si>
+    <t>Ene-2026</t>
+  </si>
+  <si>
+    <t>Feb-2026</t>
+  </si>
+  <si>
+    <t>Mar-2026</t>
+  </si>
+  <si>
+    <t>Abr-2026</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,80 +83,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -407,153 +377,127 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Mes</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Satisfacción</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Cierre</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>SLA</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Score KPI</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Nov-2025</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2">
         <v>0.58</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>0.76</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>0.49</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>0.695</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Dic-2025</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3">
         <v>0.54</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>0.75</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>0.36</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>0.6545</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Ene-2026</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4">
         <v>0.61</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>0.88</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>0.44</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>0.702</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Feb-2026</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
         <v>0.59</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>0.72</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>0.59</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>0.6355000000000001</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Mar-2026</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
         <v>0.614</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>0.675</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>0.506</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>0.61375</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.6294999999999999</v>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>0.6318</v>
+      </c>
+      <c r="C7">
+        <v>0.7354000000000001</v>
+      </c>
+      <c r="D7">
+        <v>0.31</v>
+      </c>
+      <c r="E7">
+        <v>0.6036899999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KPI_Historico actualizado - May-2026
</commit_message>
<xml_diff>
--- a/Tablas/KPI_Historico.xlsx
+++ b/Tablas/KPI_Historico.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Mes</t>
   </si>
@@ -47,6 +47,9 @@
   </si>
   <si>
     <t>Abr-2026</t>
+  </si>
+  <si>
+    <t>May-2026</t>
   </si>
 </sst>
 </file>
@@ -378,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -500,6 +503,23 @@
         <v>0.6245000000000001</v>
       </c>
     </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8">
+        <v>0.64</v>
+      </c>
+      <c r="C8">
+        <v>0.74</v>
+      </c>
+      <c r="D8">
+        <v>0.45</v>
+      </c>
+      <c r="E8">
+        <v>0.637</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
KPI_Historico actualizado - Jun-2026
</commit_message>
<xml_diff>
--- a/Tablas/KPI_Historico.xlsx
+++ b/Tablas/KPI_Historico.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Mes</t>
   </si>
@@ -50,6 +50,9 @@
   </si>
   <si>
     <t>May-2026</t>
+  </si>
+  <si>
+    <t>Jun-2026</t>
   </si>
 </sst>
 </file>
@@ -381,7 +384,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -520,6 +523,23 @@
         <v>0.635</v>
       </c>
     </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <v>0.7</v>
+      </c>
+      <c r="C9">
+        <v>0.79</v>
+      </c>
+      <c r="D9">
+        <v>0.38</v>
+      </c>
+      <c r="E9">
+        <v>0.6675</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
KPI_Historico actualizado - Jul-2026
</commit_message>
<xml_diff>
--- a/Tablas/KPI_Historico.xlsx
+++ b/Tablas/KPI_Historico.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Mes</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t>Jun-2026</t>
+  </si>
+  <si>
+    <t>Jul-2026</t>
   </si>
 </sst>
 </file>
@@ -384,7 +387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -540,6 +543,23 @@
         <v>0.6675</v>
       </c>
     </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10">
+        <v>0.67</v>
+      </c>
+      <c r="C10">
+        <v>0.76</v>
+      </c>
+      <c r="D10">
+        <v>0.44</v>
+      </c>
+      <c r="E10">
+        <v>0.6555</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
KPI_Historico actualizado - Ago-2026
</commit_message>
<xml_diff>
--- a/Tablas/KPI_Historico.xlsx
+++ b/Tablas/KPI_Historico.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Mes</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t>Jul-2026</t>
+  </si>
+  <si>
+    <t>Ago-2026</t>
   </si>
 </sst>
 </file>
@@ -387,7 +390,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -560,6 +563,23 @@
         <v>0.6555</v>
       </c>
     </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="C11">
+        <v>0.73</v>
+      </c>
+      <c r="D11">
+        <v>0.51</v>
+      </c>
+      <c r="E11">
+        <v>0.668</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
KPI_Historico: recalcular Score de Nov-2025, Dic-2025 y Ene-2026 (no surgian de 0.45*Sat+0.35*Cierre+0.20*SLA)
</commit_message>
<xml_diff>
--- a/Tablas/KPI_Historico.xlsx
+++ b/Tablas/KPI_Historico.xlsx
@@ -1,82 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>Mes</t>
-  </si>
-  <si>
-    <t>Satisfacción</t>
-  </si>
-  <si>
-    <t>Cierre</t>
-  </si>
-  <si>
-    <t>SLA</t>
-  </si>
-  <si>
-    <t>Score KPI</t>
-  </si>
-  <si>
-    <t>Nov-2025</t>
-  </si>
-  <si>
-    <t>Dic-2025</t>
-  </si>
-  <si>
-    <t>Ene-2026</t>
-  </si>
-  <si>
-    <t>Feb-2026</t>
-  </si>
-  <si>
-    <t>Mar-2026</t>
-  </si>
-  <si>
-    <t>Abr-2026</t>
-  </si>
-  <si>
-    <t>May-2026</t>
-  </si>
-  <si>
-    <t>Jun-2026</t>
-  </si>
-  <si>
-    <t>Jul-2026</t>
-  </si>
-  <si>
-    <t>Ago-2026</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -95,13 +46,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -389,194 +407,228 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Satisfacción</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Cierre</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>SLA</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Score KPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Nov-2025</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>0.58</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>0.76</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>0.49</v>
       </c>
-      <c r="E2">
-        <v>0.695</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3">
+      <c r="E2" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Dic-2025</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>0.54</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>0.75</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>0.36</v>
       </c>
-      <c r="E3">
-        <v>0.6545</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4">
+      <c r="E3" t="n">
+        <v>0.5775</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ene-2026</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>0.61</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>0.88</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>0.44</v>
       </c>
-      <c r="E4">
-        <v>0.702</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
+      <c r="E4" t="n">
+        <v>0.6705</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Feb-2026</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>0.59</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>0.72</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>0.59</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>0.6355000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Mar-2026</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>0.614</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>0.675</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>0.506</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>0.61375</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Abr-2026</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>0.63</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="n">
         <v>0.74</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>0.41</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="n">
         <v>0.6245000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>May-2026</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>0.64</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="n">
         <v>0.74</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>0.44</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="n">
         <v>0.635</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Jun-2026</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>0.7</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="n">
         <v>0.79</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>0.38</v>
       </c>
-      <c r="E9">
+      <c r="E9" t="n">
         <v>0.6675</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>0.67</v>
       </c>
-      <c r="C10">
+      <c r="C10" t="n">
         <v>0.76</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>0.44</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="n">
         <v>0.6555</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="C11">
+      <c r="C11" t="n">
         <v>0.73</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>0.51</v>
       </c>
-      <c r="E11">
+      <c r="E11" t="n">
         <v>0.668</v>
       </c>
     </row>

</xml_diff>